<commit_message>
feat(pines): importacion en modo lista por nombre de pin
</commit_message>
<xml_diff>
--- a/public/plantillas/Plantilla_Pines.xlsx
+++ b/public/plantillas/Plantilla_Pines.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Pines" sheetId="1" r:id="rId1"/>
-    <sheet name="Modo lista" sheetId="2" r:id="rId2"/>
+    <sheet name="Pines válidos" sheetId="2" r:id="rId2"/>
     <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,21 +399,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:B5"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="46.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,40 +410,7 @@
         <v>RUT</v>
       </c>
       <c r="B1" t="str">
-        <v>Semana 0/Programa IVU</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Articulación</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Voluntariado</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Proyectos Estudiantiles</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Bienestar</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Centro de Aprendizaje</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Programa de Liderazgo</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Orientación Profesional</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Estudiante Destacado/a</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Representantes Tomasin@s</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Experiencia Internacional</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Vinculación con el Medio</v>
+        <v>Pin</v>
       </c>
     </row>
     <row r="2">
@@ -462,280 +418,289 @@
         <v>12.345.678-5</v>
       </c>
       <c r="B2" t="str">
-        <v>x</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v>si</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v>1</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
-      <c r="L2" t="str">
-        <v/>
+        <v>Voluntariado</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>12.345.678-5</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Bienestar</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
         <v>9.876.543-3</v>
       </c>
-      <c r="B3" t="str">
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <v>x</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v>si</v>
-      </c>
-      <c r="F3" t="str">
-        <v>ok</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>x</v>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
+      <c r="B4" t="str">
+        <v>Semana 0/Programa IVU</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>9.876.543-3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Articulación, Programa de Liderazgo</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:A13"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>RUT</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Pines Disponibles</v>
+        <v>Nombres de pin válidos</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>12.345.678-5</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Voluntariado, Programa de Liderazgo, Bienestar</v>
+        <v>Semana 0/Programa IVU</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>9.876.543-3</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Semana 0/Programa IVU, Articulación</v>
+        <v>Articulación</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Voluntariado</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Proyectos Estudiantiles</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Bienestar</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Centro de Aprendizaje</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Programa de Liderazgo</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Orientación Profesional</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Estudiante Destacado/a</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Representantes Tomasin@s</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Experiencia Internacional</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Vinculación con el Medio</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="50.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>PLANTILLA DE IMPORTACIÓN DE PINES</v>
+        <v>PLANTILLA DE IMPORTACIÓN DE PINES (MODO LISTA)</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>⚠️ IMPORTANTE: lo que se importa son pines DISPONIBLES (por desbloquear).</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v xml:space="preserve">   No existe importación de pines ya obtenidos/entregados.</v>
+        <v>La app lee SOLO LA PRIMERA hoja ("Pines"): no cambies sus encabezados.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Cómo completarla:</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>La app lee SOLO LA PRIMERA hoja del archivo:</v>
+        <v>1. Columna RUT: el RUT del alumno (obligatorio).</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>- Hoja "Pines"           → una columna por pin (recomendado).</v>
+        <v>2. Columna Pin: escribe solo el NOMBRE del pin, sin marcar x ni números.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>- Hoja "Modo lista"      → una sola columna con los pines separados por coma.</v>
+        <v>3. Puedes repetir el mismo RUT en varias filas, un pin por fila.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Si quieres usar el modo lista, arrastra esa hoja al primer lugar del libro.</v>
+        <v>4. También puedes escribir varios pines en una celda separados por coma.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Cómo marcar un pin (modo columnas):</v>
+        <v>Ejemplos válidos:</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Escribe si, sí, x, 1, ok, true o yes en la celda.</v>
+        <v>Una fila</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Voluntariado</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Cualquier otro valor o una celda vacía significa que el pin NO se asigna.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Nombres exactos de las columnas (no los cambies):</v>
+        <v>Varios pines</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Bienestar, Articulación</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Nombre parcial</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Liderazgo</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Semana 0/Programa IVU</v>
+        <v>Nombres válidos (hoja "Pines válidos"):</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Articulación</v>
+        <v>Semana 0/Programa IVU</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Voluntariado</v>
+        <v>Articulación</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Proyectos Estudiantiles</v>
+        <v>Voluntariado</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Bienestar</v>
+        <v>Proyectos Estudiantiles</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Centro de Aprendizaje</v>
+        <v>Bienestar</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Programa de Liderazgo</v>
+        <v>Centro de Aprendizaje</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Orientación Profesional</v>
+        <v>Programa de Liderazgo</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Estudiante Destacado/a</v>
+        <v>Orientación Profesional</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Representantes Tomasin@s</v>
+        <v>Estudiante Destacado/a</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Experiencia Internacional</v>
+        <v>Representantes Tomasin@s</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>Experiencia Internacional</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>Vinculación con el Medio</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>En el modo lista puedes escribir el nombre completo o una parte:</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Ejemplo válido:</v>
-      </c>
-      <c r="B30" t="str">
-        <v>Voluntariado, Liderazgo, Bienestar</v>
+        <v>Notas:</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>- Se asignan pines DISPONIBLES (por obtener), no pines ya entregados.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>La columna RUT es obligatoria. El alumno debe existir en el sistema;</v>
+        <v>- Si el RUT no existe en el sistema, esa fila se omite.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>si el RUT no coincide con ningún estudiante, esa fila se omite.</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>Formatos permitidos: .xlsx, .xls, .csv  |  Tamaño máximo: 15 MB  |  Solo se lee la primera hoja.</v>
+        <v>- Si el nombre del pin no se reconoce, la fila se omite y se avisa en pantalla.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>- Repetir un pin ya asignado no genera duplicados.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Formatos permitidos: .xlsx, .xls, .csv  |  Tamaño máximo: 15 MB</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
se realizo plantillas de excel actualizadas para poder utilizarlas a la hora de importar
</commit_message>
<xml_diff>
--- a/public/plantillas/Plantilla_Pines.xlsx
+++ b/public/plantillas/Plantilla_Pines.xlsx
@@ -399,10 +399,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:M5"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="46.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+    <col min="9" max="9" width="26.83203125" customWidth="1"/>
+    <col min="10" max="10" width="26.83203125" customWidth="1"/>
+    <col min="11" max="11" width="26.83203125" customWidth="1"/>
+    <col min="12" max="12" width="26.83203125" customWidth="1"/>
+    <col min="13" max="13" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -410,7 +421,40 @@
         <v>RUT</v>
       </c>
       <c r="B1" t="str">
-        <v>Pin</v>
+        <v>Pin 1</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Pin 2</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Pin 3</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Pin 4</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Pin 5</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Pin 6</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Pin 7</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Pin 8</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Pin 9</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Pin 10</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Pin 11</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Pin 12</v>
       </c>
     </row>
     <row r="2">
@@ -420,287 +464,404 @@
       <c r="B2" t="str">
         <v>Voluntariado</v>
       </c>
+      <c r="C2" t="str">
+        <v>Bienestar</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>12.345.678-5</v>
+        <v>9.876.543-3</v>
       </c>
       <c r="B3" t="str">
-        <v>Bienestar</v>
+        <v>Semana 0/Programa IVU</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Articulación</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Programa de Liderazgo</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>9.876.543-3</v>
+        <v>11.222.333-4</v>
       </c>
       <c r="B4" t="str">
-        <v>Semana 0/Programa IVU</v>
+        <v>Proyectos Estudiantiles</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Centro de Aprendizaje</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Vinculación con el Medio</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>9.876.543-3</v>
+        <v>15.678.901-2</v>
       </c>
       <c r="B5" t="str">
-        <v>Articulación, Programa de Liderazgo</v>
+        <v>Orientación Profesional</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:C13"/>
   <cols>
-    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Nombres de pin válidos</v>
+        <v>Nombres de Pin Válidos</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Categoría</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Descripción</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>Semana 0/Programa IVU</v>
       </c>
+      <c r="B2" t="str">
+        <v>Inducción</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Programa de Inducción</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>Articulación</v>
       </c>
+      <c r="B3" t="str">
+        <v>Académico</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Proceso de articulación</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>Voluntariado</v>
       </c>
+      <c r="B4" t="str">
+        <v>Social</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Acción social comunitaria</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>Proyectos Estudiantiles</v>
       </c>
+      <c r="B5" t="str">
+        <v>Desarrollo</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Iniciativas y fondos</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
         <v>Bienestar</v>
       </c>
+      <c r="B6" t="str">
+        <v>Salud</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Salud mental y física</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>Centro de Aprendizaje</v>
       </c>
+      <c r="B7" t="str">
+        <v>Académico</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Apoyo y tutorías</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
         <v>Programa de Liderazgo</v>
       </c>
+      <c r="B8" t="str">
+        <v>Liderazgo</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Escuela de formación</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
         <v>Orientación Profesional</v>
       </c>
+      <c r="B9" t="str">
+        <v>Desarrollo</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Acompañamiento laboral</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
         <v>Estudiante Destacado/a</v>
       </c>
+      <c r="B10" t="str">
+        <v>Reconocimiento</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Reconocimiento al mérito</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
         <v>Representantes Tomasin@s</v>
       </c>
+      <c r="B11" t="str">
+        <v>Liderazgo</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Vocería estudiantil</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
         <v>Experiencia Internacional</v>
       </c>
+      <c r="B12" t="str">
+        <v>Desarrollo</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Intercambio y movilidad</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
         <v>Vinculación con el Medio</v>
       </c>
+      <c r="B13" t="str">
+        <v>Social</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Impacto en el entorno</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:A17"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="1" max="1" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>PLANTILLA DE IMPORTACIÓN DE PINES (MODO LISTA)</v>
+        <v>PLANTILLA DE ASIGNACIÓN DE PINES - FORMATO HORIZONTAL</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>La app lee SOLO LA PRIMERA hoja ("Pines"): no cambies sus encabezados.</v>
+        <v>Esta plantilla permite registrar los pines tomados por cada estudiante en una fila a lo largo.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Cómo completarla:</v>
+        <v>Instrucciones de llenado:</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>1. Columna RUT: el RUT del alumno (obligatorio).</v>
+        <v>1. Columna "RUT": Ingresa el RUT del alumno (con o sin puntos/guion). Debe estar previamente registrado en el sistema.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2. Columna Pin: escribe solo el NOMBRE del pin, sin marcar x ni números.</v>
+        <v>2. Columnas "Pin 1", "Pin 2", "Pin 3", etc. (a lo largo de la fila):</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>3. Puedes repetir el mismo RUT en varias filas, un pin por fila.</v>
+        <v xml:space="preserve">   - Escribe en cada cuadro/celda el nombre de UN pin que tomó el alumno.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>4. También puedes escribir varios pines en una celda separados por coma.</v>
+        <v xml:space="preserve">   - ¡No agrupes todos los pines en un solo cuadro! Cada celda corresponde a un pin individual.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v xml:space="preserve">   - Si el estudiante tomó 2 pines, completa "Pin 1" y "Pin 2" y deja las siguientes celdas vacías.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Ejemplos válidos:</v>
+        <v>3. Consulta los nombres oficiales en la pestaña "Pines válidos".</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Una fila</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Voluntariado</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Varios pines</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Bienestar, Articulación</v>
+        <v>4. El sistema reconoce nombres parciales (ejemplo: "Liderazgo" o "Voluntariado").</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Nombre parcial</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Liderazgo</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Nombres válidos (hoja "Pines válidos"):</v>
+        <v>Ejemplo de estructura:</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>RUT: 12.345.678-5  |  Pin 1: Voluntariado  |  Pin 2: Bienestar  |  Pin 3: (vacío)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Semana 0/Programa IVU</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Articulación</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Voluntariado</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Proyectos Estudiantiles</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Bienestar</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Centro de Aprendizaje</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Programa de Liderazgo</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Orientación Profesional</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Estudiante Destacado/a</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Representantes Tomasin@s</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>Experiencia Internacional</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Vinculación con el Medio</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>Notas:</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>- Se asignan pines DISPONIBLES (por obtener), no pines ya entregados.</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>- Si el RUT no existe en el sistema, esa fila se omite.</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>- Si el nombre del pin no se reconoce, la fila se omite y se avisa en pantalla.</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>- Repetir un pin ya asignado no genera duplicados.</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>Formatos permitidos: .xlsx, .xls, .csv  |  Tamaño máximo: 15 MB</v>
+        <v>Formatos soportados para importación: .xlsx, .xls, .csv</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
funcion de agregado automatico
</commit_message>
<xml_diff>
--- a/public/plantillas/Plantilla_Pines.xlsx
+++ b/public/plantillas/Plantilla_Pines.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Pines" sheetId="1" r:id="rId1"/>
+    <sheet name="Pines y Credenciales" sheetId="1" r:id="rId1"/>
     <sheet name="Pines válidos" sheetId="2" r:id="rId2"/>
     <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -399,13 +399,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:Q5"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="26.83203125" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="26.83203125" customWidth="1"/>
     <col min="7" max="7" width="26.83203125" customWidth="1"/>
     <col min="8" max="8" width="26.83203125" customWidth="1"/>
@@ -414,6 +414,10 @@
     <col min="11" max="11" width="26.83203125" customWidth="1"/>
     <col min="12" max="12" width="26.83203125" customWidth="1"/>
     <col min="13" max="13" width="26.83203125" customWidth="1"/>
+    <col min="14" max="14" width="26.83203125" customWidth="1"/>
+    <col min="15" max="15" width="26.83203125" customWidth="1"/>
+    <col min="16" max="16" width="26.83203125" customWidth="1"/>
+    <col min="17" max="17" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,39 +425,51 @@
         <v>RUT</v>
       </c>
       <c r="B1" t="str">
+        <v>Nombre</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Sede</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Lanyard</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Pasaporte</v>
+      </c>
+      <c r="F1" t="str">
         <v>Pin 1</v>
       </c>
-      <c r="C1" t="str">
+      <c r="G1" t="str">
         <v>Pin 2</v>
       </c>
-      <c r="D1" t="str">
+      <c r="H1" t="str">
         <v>Pin 3</v>
       </c>
-      <c r="E1" t="str">
+      <c r="I1" t="str">
         <v>Pin 4</v>
       </c>
-      <c r="F1" t="str">
+      <c r="J1" t="str">
         <v>Pin 5</v>
       </c>
-      <c r="G1" t="str">
+      <c r="K1" t="str">
         <v>Pin 6</v>
       </c>
-      <c r="H1" t="str">
+      <c r="L1" t="str">
         <v>Pin 7</v>
       </c>
-      <c r="I1" t="str">
+      <c r="M1" t="str">
         <v>Pin 8</v>
       </c>
-      <c r="J1" t="str">
+      <c r="N1" t="str">
         <v>Pin 9</v>
       </c>
-      <c r="K1" t="str">
+      <c r="O1" t="str">
         <v>Pin 10</v>
       </c>
-      <c r="L1" t="str">
+      <c r="P1" t="str">
         <v>Pin 11</v>
       </c>
-      <c r="M1" t="str">
+      <c r="Q1" t="str">
         <v>Pin 12</v>
       </c>
     </row>
@@ -462,23 +478,23 @@
         <v>12.345.678-5</v>
       </c>
       <c r="B2" t="str">
+        <v>Ana Rojas</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Santiago</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="F2" t="str">
         <v>Voluntariado</v>
       </c>
-      <c r="C2" t="str">
+      <c r="G2" t="str">
         <v>Bienestar</v>
       </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
@@ -495,6 +511,18 @@
         <v/>
       </c>
       <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
         <v/>
       </c>
     </row>
@@ -503,26 +531,26 @@
         <v>9.876.543-3</v>
       </c>
       <c r="B3" t="str">
+        <v>Pedro Soto</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Viña del Mar</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="F3" t="str">
         <v>Semana 0/Programa IVU</v>
       </c>
-      <c r="C3" t="str">
+      <c r="G3" t="str">
         <v>Articulación</v>
       </c>
-      <c r="D3" t="str">
+      <c r="H3" t="str">
         <v>Programa de Liderazgo</v>
       </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
       <c r="I3" t="str">
         <v/>
       </c>
@@ -536,6 +564,18 @@
         <v/>
       </c>
       <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v/>
       </c>
     </row>
@@ -544,26 +584,26 @@
         <v>11.222.333-4</v>
       </c>
       <c r="B4" t="str">
+        <v>Claudia Morales</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Concepción</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="F4" t="str">
         <v>Proyectos Estudiantiles</v>
       </c>
-      <c r="C4" t="str">
+      <c r="G4" t="str">
         <v>Centro de Aprendizaje</v>
       </c>
-      <c r="D4" t="str">
+      <c r="H4" t="str">
         <v>Vinculación con el Medio</v>
       </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
       <c r="I4" t="str">
         <v/>
       </c>
@@ -577,6 +617,18 @@
         <v/>
       </c>
       <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
         <v/>
       </c>
     </row>
@@ -585,20 +637,20 @@
         <v>15.678.901-2</v>
       </c>
       <c r="B5" t="str">
+        <v>Felipe Araya</v>
+      </c>
+      <c r="C5" t="str">
+        <v>La Serena</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="F5" t="str">
         <v>Orientación Profesional</v>
       </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
       <c r="G5" t="str">
         <v/>
       </c>
@@ -618,12 +670,24 @@
         <v/>
       </c>
       <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -789,19 +853,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A16"/>
   <cols>
-    <col min="1" max="1" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="95.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>PLANTILLA DE ASIGNACIÓN DE PINES - FORMATO HORIZONTAL</v>
+        <v>PLANTILLA DE LLENADO AUTOMÁTICO DE PINES, LANYARD Y PASAPORTE</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Esta plantilla permite registrar los pines tomados por cada estudiante en una fila a lo largo.</v>
+        <v>Esta plantilla permite registrar y actualizar pines y credenciales para estudiantes de UNA O VARIAS SEDES a la vez.</v>
       </c>
     </row>
     <row r="5">
@@ -811,57 +875,57 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>1. Columna "RUT": Ingresa el RUT del alumno (con o sin puntos/guion). Debe estar previamente registrado en el sistema.</v>
+        <v>1. Columna "RUT": Ingresa el RUT del alumno (con o sin puntos/guion).</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2. Columnas "Pin 1", "Pin 2", "Pin 3", etc. (a lo largo de la fila):</v>
+        <v>2. Columna "Nombre" (opcional): Nombre del alumno.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v xml:space="preserve">   - Escribe en cada cuadro/celda el nombre de UN pin que tomó el alumno.</v>
+        <v>3. Columna "Sede" (opcional): Sede a la que pertenece el alumno (permite mezclar varias sedes en el mismo archivo).</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v xml:space="preserve">   - ¡No agrupes todos los pines en un solo cuadro! Cada celda corresponde a un pin individual.</v>
+        <v>4. Columnas "Lanyard" y "Pasaporte": Escribe "Sí", "X", "1" o "Entregado" si se le entregó la credencial (o deja vacío si no).</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v xml:space="preserve">   - Si el estudiante tomó 2 pines, completa "Pin 1" y "Pin 2" y deja las siguientes celdas vacías.</v>
+        <v>5. Columnas "Pin 1", "Pin 2", "Pin 3", etc. (a lo largo de la fila):</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>3. Consulta los nombres oficiales en la pestaña "Pines válidos".</v>
+        <v xml:space="preserve">   - Escribe en cada cuadro/celda el nombre de UN pin que ganó o tomó el estudiante.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>4. El sistema reconoce nombres parciales (ejemplo: "Liderazgo" o "Voluntariado").</v>
+        <v xml:space="preserve">   - ¡No agrupes todos los pines en un solo cuadro! Cada celda corresponde a un pin individual.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v xml:space="preserve">   - Si el estudiante tomó 2 pines, completa "Pin 1" y "Pin 2" y deja las siguientes celdas vacías.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Ejemplo de estructura:</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>RUT: 12.345.678-5  |  Pin 1: Voluntariado  |  Pin 2: Bienestar  |  Pin 3: (vacío)</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
+        <v>6. Consulta los nombres oficiales en la pestaña "Pines válidos". Se aceptan nombres parciales (ejemplo: "Liderazgo" o "Voluntariado").</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>Formatos soportados para importación: .xlsx, .xls, .csv</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>